<commit_message>
Update Selenium test to generate professional Excel report and add to workflow
</commit_message>
<xml_diff>
--- a/test cases/see secrity test_Selenium.xlsx
+++ b/test cases/see secrity test_Selenium.xlsx
@@ -40,7 +40,7 @@
     <t>Selenium: wait for accessibility id 'Login Screen'</t>
   </si>
   <si>
-    <t>2026-06-17 09:12:20</t>
+    <t>2026-06-18 03:01:08</t>
   </si>
   <si>
     <t>Verify splash routes to dashboard for authenticated users</t>
@@ -487,7 +487,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -495,13 +495,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,1702 +877,1702 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="C18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C22" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="C22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="C23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="C24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C25" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="C25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="C26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="A27" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C27" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C28" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="C28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C29" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="C29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C30" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C30" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C31" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C32" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C32" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C33" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="A34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C34" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="A35" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C35" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="C35" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="A36" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C36" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="C36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="A37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C37" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="C37" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" t="s">
+      <c r="A38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C38" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="C38" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="C39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="A40" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C40" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="C40" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="A41" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C41" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="C41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>20</v>
-      </c>
-      <c r="B42" t="s">
+      <c r="A42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C42" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="C42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C43" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="A44" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C44" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="C44" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="A45" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C45" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="C45" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>20</v>
-      </c>
-      <c r="B46" t="s">
+      <c r="A46" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C46" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="C46" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="A47" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C47" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="C47" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="A48" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C48" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="C48" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+      <c r="A49" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C49" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49" t="s">
+      <c r="C49" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B50" t="s">
+      <c r="A50" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C50" t="s">
-        <v>7</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="C50" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="A51" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C51" t="s">
-        <v>7</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="C51" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="A52" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C52" t="s">
-        <v>7</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="C52" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="A53" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C53" t="s">
-        <v>7</v>
-      </c>
-      <c r="D53" t="s">
+      <c r="C53" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" t="s">
+      <c r="A54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C54" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" t="s">
+      <c r="C54" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E54" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="A55" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C55" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="C55" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E55" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="A56" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C56" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" t="s">
+      <c r="C56" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+      <c r="A57" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C57" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="C57" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E57" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>20</v>
-      </c>
-      <c r="B58" t="s">
+      <c r="A58" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C58" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58" t="s">
+      <c r="C58" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="A59" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59" t="s">
+      <c r="C59" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E59" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C60" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" t="s">
+      <c r="C60" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E60" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="A61" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C61" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61" t="s">
+      <c r="C61" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>20</v>
-      </c>
-      <c r="B62" t="s">
+      <c r="A62" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C62" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62" t="s">
+      <c r="C62" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E62" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+      <c r="A63" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C63" t="s">
-        <v>7</v>
-      </c>
-      <c r="D63" t="s">
+      <c r="C63" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E63" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="A64" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C64" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" t="s">
+      <c r="C64" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E64" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+      <c r="A65" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C65" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="C65" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E65" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>20</v>
-      </c>
-      <c r="B66" t="s">
+      <c r="A66" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C66" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" t="s">
+      <c r="C66" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E66" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+      <c r="A67" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C67" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" t="s">
+      <c r="C67" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E67" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+      <c r="A68" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C68" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68" t="s">
+      <c r="C68" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E68" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+      <c r="A69" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C69" t="s">
-        <v>7</v>
-      </c>
-      <c r="D69" t="s">
+      <c r="C69" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E69" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>20</v>
-      </c>
-      <c r="B70" t="s">
+      <c r="A70" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C70" t="s">
-        <v>7</v>
-      </c>
-      <c r="D70" t="s">
+      <c r="C70" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E70" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="A71" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C71" t="s">
-        <v>7</v>
-      </c>
-      <c r="D71" t="s">
+      <c r="C71" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E71" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="A72" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C72" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" t="s">
+      <c r="C72" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E72" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="A73" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C73" t="s">
-        <v>7</v>
-      </c>
-      <c r="D73" t="s">
+      <c r="C73" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E73" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>20</v>
-      </c>
-      <c r="B74" t="s">
+      <c r="A74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C74" t="s">
-        <v>7</v>
-      </c>
-      <c r="D74" t="s">
+      <c r="C74" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E74" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+      <c r="A75" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C75" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" t="s">
+      <c r="C75" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E75" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="A76" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C76" t="s">
-        <v>7</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="C76" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E76" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="A77" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C77" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" t="s">
+      <c r="C77" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E77" t="s">
+      <c r="E77" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>20</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="A78" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C78" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="C78" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E78" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+      <c r="A79" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C79" t="s">
-        <v>7</v>
-      </c>
-      <c r="D79" t="s">
+      <c r="C79" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E79" t="s">
+      <c r="E79" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+      <c r="A80" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C80" t="s">
-        <v>7</v>
-      </c>
-      <c r="D80" t="s">
+      <c r="C80" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E80" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+      <c r="A81" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C81" t="s">
-        <v>7</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="C81" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E81" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>20</v>
-      </c>
-      <c r="B82" t="s">
+      <c r="A82" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C82" t="s">
-        <v>7</v>
-      </c>
-      <c r="D82" t="s">
+      <c r="C82" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E82" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+      <c r="A83" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C83" t="s">
-        <v>7</v>
-      </c>
-      <c r="D83" t="s">
+      <c r="C83" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E83" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="A84" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C84" t="s">
-        <v>7</v>
-      </c>
-      <c r="D84" t="s">
+      <c r="C84" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E84" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+      <c r="A85" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C85" t="s">
-        <v>7</v>
-      </c>
-      <c r="D85" t="s">
+      <c r="C85" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E85" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>20</v>
-      </c>
-      <c r="B86" t="s">
+      <c r="A86" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C86" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" t="s">
+      <c r="C86" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E86" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="A87" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C87" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" t="s">
+      <c r="C87" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E87" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="A88" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C88" t="s">
-        <v>7</v>
-      </c>
-      <c r="D88" t="s">
+      <c r="C88" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E88" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="A89" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C89" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" t="s">
+      <c r="C89" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E89" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>20</v>
-      </c>
-      <c r="B90" t="s">
+      <c r="A90" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C90" t="s">
-        <v>7</v>
-      </c>
-      <c r="D90" t="s">
+      <c r="C90" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E90" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+      <c r="A91" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C91" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" t="s">
+      <c r="C91" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E91" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="A92" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C92" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" t="s">
+      <c r="C92" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E92" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+      <c r="A93" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C93" t="s">
-        <v>7</v>
-      </c>
-      <c r="D93" t="s">
+      <c r="C93" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E93" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>20</v>
-      </c>
-      <c r="B94" t="s">
+      <c r="A94" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C94" t="s">
-        <v>7</v>
-      </c>
-      <c r="D94" t="s">
+      <c r="C94" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E94" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+      <c r="A95" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C95" t="s">
-        <v>7</v>
-      </c>
-      <c r="D95" t="s">
+      <c r="C95" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E95" t="s">
+      <c r="E95" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+      <c r="A96" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C96" t="s">
-        <v>7</v>
-      </c>
-      <c r="D96" t="s">
+      <c r="C96" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E96" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+      <c r="A97" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C97" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" t="s">
+      <c r="C97" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E97" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>20</v>
-      </c>
-      <c r="B98" t="s">
+      <c r="A98" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B98" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C98" t="s">
-        <v>7</v>
-      </c>
-      <c r="D98" t="s">
+      <c r="C98" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E98" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="A99" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C99" t="s">
-        <v>7</v>
-      </c>
-      <c r="D99" t="s">
+      <c r="C99" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D99" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E99" t="s">
+      <c r="E99" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+      <c r="A100" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C100" t="s">
-        <v>7</v>
-      </c>
-      <c r="D100" t="s">
+      <c r="C100" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D100" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E100" t="s">
+      <c r="E100" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+      <c r="A101" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C101" t="s">
-        <v>7</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="C101" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D101" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E101" s="2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Supabase tracking features
</commit_message>
<xml_diff>
--- a/test cases/see secrity test_Selenium.xlsx
+++ b/test cases/see secrity test_Selenium.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D4BE90BB10EF6E7487D848052437F4A84CB94588" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Selenium E2E Screen Tests" state="visible" r:id="rId4"/>
+    <sheet name="Selenium E2E Screen Tests" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -460,18 +464,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -496,10 +502,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -848,9 +862,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E101"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -859,7 +873,7 @@
     <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -876,7 +890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -893,7 +907,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -910,7 +924,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -927,7 +941,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -944,7 +958,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -961,7 +975,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -978,7 +992,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -995,7 +1009,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -1012,7 +1026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -1029,7 +1043,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -1046,7 +1060,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -1063,7 +1077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1080,7 +1094,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1097,7 +1111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1114,7 +1128,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1131,7 +1145,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1148,7 +1162,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1165,7 +1179,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
@@ -1182,7 +1196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>41</v>
       </c>
@@ -1199,7 +1213,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
@@ -1216,7 +1230,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>41</v>
       </c>
@@ -1233,7 +1247,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
@@ -1250,7 +1264,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>41</v>
       </c>
@@ -1267,7 +1281,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>41</v>
       </c>
@@ -1284,7 +1298,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>58</v>
       </c>
@@ -1301,7 +1315,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>58</v>
       </c>
@@ -1318,7 +1332,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>58</v>
       </c>
@@ -1335,7 +1349,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>5</v>
       </c>
@@ -1352,7 +1366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -1369,7 +1383,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>41</v>
       </c>
@@ -1386,7 +1400,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>58</v>
       </c>
@@ -1403,7 +1417,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>5</v>
       </c>
@@ -1420,7 +1434,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -1437,7 +1451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>41</v>
       </c>
@@ -1454,7 +1468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>58</v>
       </c>
@@ -1471,7 +1485,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>5</v>
       </c>
@@ -1488,7 +1502,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -1505,7 +1519,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
@@ -1522,7 +1536,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>58</v>
       </c>
@@ -1539,7 +1553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>5</v>
       </c>
@@ -1556,7 +1570,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -1573,7 +1587,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -1590,7 +1604,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>58</v>
       </c>
@@ -1607,7 +1621,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>5</v>
       </c>
@@ -1624,7 +1638,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -1641,7 +1655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>41</v>
       </c>
@@ -1658,7 +1672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>58</v>
       </c>
@@ -1675,7 +1689,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>5</v>
       </c>
@@ -1692,7 +1706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -1709,7 +1723,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>41</v>
       </c>
@@ -1726,7 +1740,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>58</v>
       </c>
@@ -1743,7 +1757,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>5</v>
       </c>
@@ -1760,7 +1774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>20</v>
       </c>
@@ -1777,7 +1791,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>41</v>
       </c>
@@ -1794,7 +1808,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>58</v>
       </c>
@@ -1811,7 +1825,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>5</v>
       </c>
@@ -1828,7 +1842,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>20</v>
       </c>
@@ -1845,7 +1859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>41</v>
       </c>
@@ -1862,7 +1876,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
@@ -1879,7 +1893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>5</v>
       </c>
@@ -1896,7 +1910,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>20</v>
       </c>
@@ -1913,7 +1927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>41</v>
       </c>
@@ -1930,7 +1944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>58</v>
       </c>
@@ -1947,7 +1961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>5</v>
       </c>
@@ -1964,7 +1978,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>20</v>
       </c>
@@ -1981,7 +1995,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>41</v>
       </c>
@@ -1998,7 +2012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>58</v>
       </c>
@@ -2015,7 +2029,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>5</v>
       </c>
@@ -2032,7 +2046,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>20</v>
       </c>
@@ -2049,7 +2063,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>41</v>
       </c>
@@ -2066,7 +2080,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>58</v>
       </c>
@@ -2083,7 +2097,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>5</v>
       </c>
@@ -2100,7 +2114,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>20</v>
       </c>
@@ -2117,7 +2131,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>41</v>
       </c>
@@ -2134,7 +2148,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>58</v>
       </c>
@@ -2151,7 +2165,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>5</v>
       </c>
@@ -2168,7 +2182,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>20</v>
       </c>
@@ -2185,7 +2199,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>41</v>
       </c>
@@ -2202,7 +2216,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>58</v>
       </c>
@@ -2219,7 +2233,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>5</v>
       </c>
@@ -2236,7 +2250,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>20</v>
       </c>
@@ -2253,7 +2267,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>41</v>
       </c>
@@ -2270,7 +2284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>58</v>
       </c>
@@ -2287,7 +2301,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>5</v>
       </c>
@@ -2304,7 +2318,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>20</v>
       </c>
@@ -2321,7 +2335,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>41</v>
       </c>
@@ -2338,7 +2352,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>58</v>
       </c>
@@ -2355,7 +2369,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>5</v>
       </c>
@@ -2372,7 +2386,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>20</v>
       </c>
@@ -2389,7 +2403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>41</v>
       </c>
@@ -2406,7 +2420,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>58</v>
       </c>
@@ -2423,7 +2437,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>5</v>
       </c>
@@ -2440,7 +2454,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>20</v>
       </c>
@@ -2457,7 +2471,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>41</v>
       </c>
@@ -2474,7 +2488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>58</v>
       </c>
@@ -2491,7 +2505,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>5</v>
       </c>
@@ -2508,7 +2522,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>20</v>
       </c>
@@ -2525,7 +2539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>41</v>
       </c>
@@ -2542,7 +2556,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>58</v>
       </c>
@@ -2559,7 +2573,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>5</v>
       </c>
@@ -2578,6 +2592,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>